<commit_message>
Ajustes de redaccion en analisis, conclusiones y matriz IREB
</commit_message>
<xml_diff>
--- a/Unidad 1/G5_Matriz_IREB_V3.0.xlsx
+++ b/Unidad 1/G5_Matriz_IREB_V3.0.xlsx
@@ -887,13 +887,14 @@
     <t>Realizable</t>
   </si>
   <si>
-    <t>1. Funcionalidad tomada en cuenta dentro de la estimación del costo del proyecto (900$)
-2. No se ha desarrollado</t>
+    <t>1. Funcionalidad considerada en la estimación del proyecto (144 horas por integrante, costeo por hora según el rol).
+2. Tecnologías y hardware mínimo definidos en la ERS (secciones 3.1.6 a 3.1.11): React + Vite, Node.js con Express, servicios REST con JSON.
+3. Su construcción está planificada para las fases posteriores al análisis y diseño.</t>
   </si>
   <si>
     <t>1. Funcionalidad considerada en la estimación del proyecto (144 horas por integrante, costeo por hora según el rol).
 2. Tecnologías y hardware mínimo definidos en la ERS (secciones 3.1.6 a 3.1.11): React + Vite, Node.js con Express, servicios REST con JSON.
-3. Aún no se ha desarrollado.</t>
+3. Su construcción está planificada para las fases posteriores al análisis y diseño.</t>
   </si>
   <si>
     <t>Traceable</t>

</xml_diff>